<commit_message>
Fix the rounding error issue in LowDepthQAE. Add results.
</commit_message>
<xml_diff>
--- a/Result/DivideRBM_RQAE_eps0=2^-10_R=12_maxdeg=5_integEpsabs=1e-4.xlsx
+++ b/Result/DivideRBM_RQAE_eps0=2^-10_R=12_maxdeg=5_integEpsabs=1e-4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koich\Desktop\Code\DivQCOSDE\Result\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBA0FB6-E59A-4B3E-8369-1473365C3B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7329BAD6-2DED-4D66-9A57-495CD977849F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1215" yWindow="1215" windowWidth="18390" windowHeight="9015" xr2:uid="{DDFBC754-980A-4BFD-AE2C-311ED991EAD0}"/>
+    <workbookView xWindow="345" yWindow="1635" windowWidth="18390" windowHeight="9015" xr2:uid="{DDFBC754-980A-4BFD-AE2C-311ED991EAD0}"/>
   </bookViews>
   <sheets>
     <sheet name="RQAE_eps0=2^-10_R=12_deg10" sheetId="1" r:id="rId1"/>
@@ -111,9 +111,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="176" formatCode="0.00000"/>
     <numFmt numFmtId="177" formatCode="0.000000"/>
+    <numFmt numFmtId="178" formatCode="#,##0.0000;[Red]\-#,##0.0000"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -704,7 +705,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -721,6 +722,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3292,6 +3296,8 @@
         <f t="shared" si="2"/>
         <v>4094</v>
       </c>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
       <c r="Q4" s="3">
         <f t="shared" si="3"/>
         <v>97478260.605840072</v>
@@ -3346,6 +3352,8 @@
         <f t="shared" si="2"/>
         <v>4801.8</v>
       </c>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
       <c r="Q5" s="3">
         <f t="shared" si="3"/>
         <v>46476653.164291337</v>
@@ -3400,6 +3408,8 @@
         <f t="shared" si="2"/>
         <v>5792</v>
       </c>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
       <c r="Q6" s="3">
         <f t="shared" si="3"/>
         <v>70601831.171514302</v>
@@ -3454,6 +3464,8 @@
         <f t="shared" si="2"/>
         <v>6867.9</v>
       </c>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
       <c r="Q7" s="3">
         <f t="shared" si="3"/>
         <v>239878645.15635109</v>
@@ -3508,6 +3520,8 @@
         <f t="shared" si="2"/>
         <v>8190.3</v>
       </c>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
       <c r="Q8" s="3">
         <f t="shared" si="3"/>
         <v>91912539.122116357</v>

</xml_diff>